<commit_message>
Update to saf case study
</commit_message>
<xml_diff>
--- a/src/technology/sustainable-aviation-fuel/saf.xlsx
+++ b/src/technology/sustainable-aviation-fuel/saf.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10212"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10414"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tghosh/Library/CloudStorage/OneDrive-NREL/work_NREL/tyche/src/technology/sustainable-aviation-fuel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nrel-my.sharepoint.com/personal/tghosh_nrel_gov/Documents/work_NREL/tyche/tyche/src/technology/sustainable-aviation-fuel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFEDA073-76B4-0D4A-A9EF-AFDEAC405683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{BFEDA073-76B4-0D4A-A9EF-AFDEAC405683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F20BCBA-BCF1-3148-B7BA-8B683E6927E4}"/>
   <bookViews>
-    <workbookView xWindow="12600" yWindow="5960" windowWidth="38600" windowHeight="19040" activeTab="2" xr2:uid="{021BDB00-52DC-4A4E-ACEA-9258FAE2C700}"/>
+    <workbookView xWindow="46980" yWindow="3060" windowWidth="34560" windowHeight="19040" activeTab="4" xr2:uid="{021BDB00-52DC-4A4E-ACEA-9258FAE2C700}"/>
   </bookViews>
   <sheets>
     <sheet name="designs" sheetId="1" r:id="rId1"/>
@@ -42,14 +42,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="73">
   <si>
     <t>Technology</t>
   </si>
   <si>
-    <t>Scenario</t>
-  </si>
-  <si>
     <t>Variable</t>
   </si>
   <si>
@@ -258,6 +255,12 @@
   </si>
   <si>
     <t>vb</t>
+  </si>
+  <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>st.triang(1, loc=46.5, scale=0.00001)</t>
   </si>
 </sst>
 </file>
@@ -314,9 +317,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -354,7 +357,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -460,7 +463,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -602,7 +605,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -625,988 +628,1156 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
         <v>42</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>43</v>
       </c>
       <c r="E2">
         <v>3680</v>
       </c>
+      <c r="F2" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
         <v>42</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>43</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
+      <c r="F3" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
+      <c r="F4" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
+      <c r="F5" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" t="s">
         <v>7</v>
-      </c>
-      <c r="D6" t="s">
-        <v>8</v>
       </c>
       <c r="E6">
         <v>7365</v>
       </c>
+      <c r="F6" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
+      <c r="F7" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E8">
         <v>1</v>
       </c>
+      <c r="F8" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
+      <c r="F9" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
         <v>42</v>
-      </c>
-      <c r="C10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" t="s">
-        <v>43</v>
       </c>
       <c r="E10">
         <f>114/1000</f>
         <v>0.114</v>
       </c>
+      <c r="F10" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E11">
         <v>0.5</v>
       </c>
+      <c r="F11" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E12">
         <f>0.22/1000</f>
         <v>2.2000000000000001E-4</v>
       </c>
+      <c r="F12" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E13">
         <v>4.41</v>
       </c>
+      <c r="F13" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E14">
         <v>20</v>
       </c>
+      <c r="F14" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E15">
         <v>20</v>
       </c>
+      <c r="F15" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E16">
-        <v>3680</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+        <v>3500</v>
+      </c>
+      <c r="F16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E17">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F17" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D19" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" t="s">
         <v>7</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20">
+        <v>7100</v>
+      </c>
+      <c r="F20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" t="s">
         <v>8</v>
       </c>
-      <c r="E20">
-        <v>7365</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>41</v>
-      </c>
-      <c r="B21" t="s">
-        <v>44</v>
-      </c>
-      <c r="C21" t="s">
-        <v>9</v>
-      </c>
       <c r="D21" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F21" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" t="s">
         <v>44</v>
-      </c>
-      <c r="C22" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" t="s">
-        <v>45</v>
       </c>
       <c r="E22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F22" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C23" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F23" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D24" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E24">
         <f>114/1000</f>
         <v>0.114</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F24" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B25" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E25">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F25" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B26" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D26" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E26">
         <f>0.22/1000</f>
         <v>2.2000000000000001E-4</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F26" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B27" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" t="s">
         <v>44</v>
-      </c>
-      <c r="C27" t="s">
-        <v>14</v>
-      </c>
-      <c r="D27" t="s">
-        <v>45</v>
       </c>
       <c r="E27">
         <v>4.41</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F27" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B28" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C28" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E28">
         <v>20</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F28" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B29" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C29" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D29" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E29">
         <v>20</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F29" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B30" t="s">
+        <v>41</v>
+      </c>
+      <c r="C30" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" t="s">
         <v>42</v>
-      </c>
-      <c r="C30" t="s">
-        <v>7</v>
-      </c>
-      <c r="D30" t="s">
-        <v>43</v>
       </c>
       <c r="E30">
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F30" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B31" t="s">
+        <v>41</v>
+      </c>
+      <c r="C31" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" t="s">
         <v>42</v>
-      </c>
-      <c r="C31" t="s">
-        <v>9</v>
-      </c>
-      <c r="D31" t="s">
-        <v>43</v>
       </c>
       <c r="E31">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F31" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C32" t="s">
+        <v>6</v>
+      </c>
+      <c r="D32" t="s">
         <v>65</v>
-      </c>
-      <c r="B32" t="s">
-        <v>42</v>
-      </c>
-      <c r="C32" t="s">
-        <v>7</v>
-      </c>
-      <c r="D32" t="s">
-        <v>66</v>
       </c>
       <c r="E32">
         <v>2680</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F32" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" t="s">
+        <v>41</v>
+      </c>
+      <c r="C33" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" t="s">
         <v>65</v>
-      </c>
-      <c r="B33" t="s">
-        <v>42</v>
-      </c>
-      <c r="C33" t="s">
-        <v>9</v>
-      </c>
-      <c r="D33" t="s">
-        <v>66</v>
       </c>
       <c r="E33">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F33" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B34" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C34" t="s">
+        <v>6</v>
+      </c>
+      <c r="D34" t="s">
         <v>7</v>
-      </c>
-      <c r="D34" t="s">
-        <v>8</v>
       </c>
       <c r="E34">
         <v>7365</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F34" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B35" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C35" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E35">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F35" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C36" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D36" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E36">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F36" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B37" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C37" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D37" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E37">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F37" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B38" t="s">
+        <v>41</v>
+      </c>
+      <c r="C38" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38" t="s">
         <v>42</v>
-      </c>
-      <c r="C38" t="s">
-        <v>13</v>
-      </c>
-      <c r="D38" t="s">
-        <v>43</v>
       </c>
       <c r="E38">
         <f>114/1000</f>
         <v>0.114</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F38" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" t="s">
+        <v>41</v>
+      </c>
+      <c r="C39" t="s">
+        <v>12</v>
+      </c>
+      <c r="D39" t="s">
         <v>65</v>
-      </c>
-      <c r="B39" t="s">
-        <v>42</v>
-      </c>
-      <c r="C39" t="s">
-        <v>13</v>
-      </c>
-      <c r="D39" t="s">
-        <v>66</v>
       </c>
       <c r="E39">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F39" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C40" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E40">
         <f>0.22/1000</f>
         <v>2.2000000000000001E-4</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F40" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C41" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D41" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E41">
         <v>4.41</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F41" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C42" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D42" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E42">
         <v>20</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F42" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C43" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D43" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E43">
         <v>20</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B44" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C44" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D44" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E44">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F44" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B45" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C45" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D45" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E45">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F45" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
+        <v>64</v>
+      </c>
+      <c r="B46" t="s">
+        <v>43</v>
+      </c>
+      <c r="C46" t="s">
+        <v>6</v>
+      </c>
+      <c r="D46" t="s">
         <v>65</v>
       </c>
-      <c r="B46" t="s">
-        <v>44</v>
-      </c>
-      <c r="C46" t="s">
-        <v>7</v>
-      </c>
-      <c r="D46" t="s">
-        <v>66</v>
-      </c>
       <c r="E46">
-        <v>2680</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+        <v>2500</v>
+      </c>
+      <c r="F46" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
+        <v>64</v>
+      </c>
+      <c r="B47" t="s">
+        <v>43</v>
+      </c>
+      <c r="C47" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" t="s">
         <v>65</v>
-      </c>
-      <c r="B47" t="s">
-        <v>44</v>
-      </c>
-      <c r="C47" t="s">
-        <v>9</v>
-      </c>
-      <c r="D47" t="s">
-        <v>66</v>
       </c>
       <c r="E47">
         <v>1</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F47" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B48" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C48" t="s">
+        <v>6</v>
+      </c>
+      <c r="D48" t="s">
         <v>7</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48">
+        <v>7000</v>
+      </c>
+      <c r="F48" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>64</v>
+      </c>
+      <c r="B49" t="s">
+        <v>43</v>
+      </c>
+      <c r="C49" t="s">
         <v>8</v>
       </c>
-      <c r="E48">
-        <v>7365</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>65</v>
-      </c>
-      <c r="B49" t="s">
-        <v>44</v>
-      </c>
-      <c r="C49" t="s">
-        <v>9</v>
-      </c>
       <c r="D49" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E49">
         <v>1</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F49" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B50" t="s">
+        <v>43</v>
+      </c>
+      <c r="C50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D50" t="s">
         <v>44</v>
-      </c>
-      <c r="C50" t="s">
-        <v>10</v>
-      </c>
-      <c r="D50" t="s">
-        <v>45</v>
       </c>
       <c r="E50">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F50" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B51" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C51" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D51" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E51">
         <v>1</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F51" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B52" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C52" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D52" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E52">
         <f>114/1000</f>
         <v>0.114</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F52" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
+        <v>64</v>
+      </c>
+      <c r="B53" t="s">
+        <v>43</v>
+      </c>
+      <c r="C53" t="s">
+        <v>12</v>
+      </c>
+      <c r="D53" t="s">
         <v>65</v>
-      </c>
-      <c r="B53" t="s">
-        <v>44</v>
-      </c>
-      <c r="C53" t="s">
-        <v>13</v>
-      </c>
-      <c r="D53" t="s">
-        <v>66</v>
       </c>
       <c r="E53">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F53" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C54" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D54" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E54">
         <f>0.22/1000</f>
         <v>2.2000000000000001E-4</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F54" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B55" t="s">
+        <v>43</v>
+      </c>
+      <c r="C55" t="s">
+        <v>13</v>
+      </c>
+      <c r="D55" t="s">
         <v>44</v>
-      </c>
-      <c r="C55" t="s">
-        <v>14</v>
-      </c>
-      <c r="D55" t="s">
-        <v>45</v>
       </c>
       <c r="E55">
         <v>4.41</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F55" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B56" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C56" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D56" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E56">
         <v>20</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F56" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B57" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C57" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D57" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E57">
         <v>20</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F57" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="E63" s="1"/>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="E64" s="1"/>
     </row>
     <row r="65" spans="5:5" x14ac:dyDescent="0.2">
@@ -1634,30 +1805,30 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
         <v>26</v>
       </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>27</v>
       </c>
-      <c r="E1" t="s">
-        <v>28</v>
-      </c>
       <c r="F1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -1665,13 +1836,13 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -1679,13 +1850,13 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -1693,58 +1864,61 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>66</v>
+        <v>30</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="E7" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
         <v>31</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="s">
         <v>31</v>
@@ -1752,47 +1926,44 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
         <v>32</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="D10">
-        <v>2</v>
-      </c>
-      <c r="E10" t="s">
-        <v>34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D11">
         <v>0</v>
@@ -1800,13 +1971,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1814,13 +1985,13 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -1828,13 +1999,13 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="B14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" t="s">
         <v>7</v>
-      </c>
-      <c r="C14" t="s">
-        <v>8</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -1842,13 +2013,13 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s">
         <v>65</v>
-      </c>
-      <c r="B15" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" t="s">
-        <v>66</v>
       </c>
       <c r="D15">
         <v>2</v>
@@ -1856,30 +2027,33 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="B16" t="s">
         <v>29</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
+      <c r="E16" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C17" t="s">
         <v>31</v>
       </c>
       <c r="D17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" t="s">
         <v>31</v>
@@ -1887,39 +2061,39 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C18" t="s">
         <v>32</v>
       </c>
       <c r="D18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C19" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="D19">
-        <v>2</v>
-      </c>
-      <c r="E19" t="s">
-        <v>34</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F19">
+    <sortCondition ref="A1:A19"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1938,71 +2112,71 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" t="s">
         <v>15</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>16</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>17</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>18</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>19</v>
       </c>
-      <c r="G1" t="s">
-        <v>20</v>
-      </c>
       <c r="H1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D2" t="s">
         <v>21</v>
       </c>
-      <c r="C2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>22</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>23</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>24</v>
-      </c>
-      <c r="G2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" t="s">
         <v>21</v>
       </c>
-      <c r="C3" t="s">
-        <v>67</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>22</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>23</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>24</v>
-      </c>
-      <c r="G3" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -2022,60 +2196,60 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" t="s">
         <v>35</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>36</v>
       </c>
-      <c r="C1" t="s">
-        <v>37</v>
-      </c>
       <c r="D1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" t="s">
         <v>68</v>
-      </c>
-      <c r="C4" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2090,7 +2264,7 @@
   <cols>
     <col min="3" max="3" width="19.6640625" customWidth="1"/>
     <col min="4" max="4" width="12.1640625" customWidth="1"/>
-    <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -2098,33 +2272,33 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -2133,18 +2307,18 @@
         <v>111000000</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -2154,18 +2328,18 @@
         <v>62160000</v>
       </c>
       <c r="F3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D4">
         <v>2</v>
@@ -2174,38 +2348,38 @@
         <v>0.17219999999999999</v>
       </c>
       <c r="F4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D5">
         <v>3</v>
       </c>
-      <c r="E5">
-        <v>43.5</v>
+      <c r="E5" t="s">
+        <v>72</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D6">
         <v>4</v>
@@ -2214,18 +2388,18 @@
         <v>68</v>
       </c>
       <c r="F6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D7">
         <v>5</v>
@@ -2234,18 +2408,18 @@
         <v>1000</v>
       </c>
       <c r="F7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -2254,18 +2428,18 @@
         <v>111000000</v>
       </c>
       <c r="F8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -2275,18 +2449,18 @@
         <v>62160000</v>
       </c>
       <c r="F9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D10">
         <v>2</v>
@@ -2295,38 +2469,38 @@
         <v>0.17219999999999999</v>
       </c>
       <c r="F10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D11">
         <v>3</v>
       </c>
-      <c r="E11">
-        <v>43.5</v>
+      <c r="E11" t="s">
+        <v>72</v>
       </c>
       <c r="F11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D12">
         <v>4</v>
@@ -2335,18 +2509,18 @@
         <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D13">
         <v>5</v>
@@ -2355,18 +2529,18 @@
         <v>1000</v>
       </c>
       <c r="F13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -2375,18 +2549,18 @@
         <v>111000000</v>
       </c>
       <c r="F14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -2396,18 +2570,18 @@
         <v>62160000</v>
       </c>
       <c r="F15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D16">
         <v>2</v>
@@ -2416,38 +2590,38 @@
         <v>0.17219999999999999</v>
       </c>
       <c r="F16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D17">
         <v>3</v>
       </c>
-      <c r="E17">
-        <v>43.5</v>
+      <c r="E17" t="s">
+        <v>72</v>
       </c>
       <c r="F17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D18">
         <v>4</v>
@@ -2456,18 +2630,18 @@
         <v>68</v>
       </c>
       <c r="F18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D19">
         <v>5</v>
@@ -2476,18 +2650,18 @@
         <v>1000</v>
       </c>
       <c r="F19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -2496,18 +2670,18 @@
         <v>111000000</v>
       </c>
       <c r="F20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -2517,18 +2691,18 @@
         <v>62160000</v>
       </c>
       <c r="F21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C22" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D22">
         <v>2</v>
@@ -2537,38 +2711,38 @@
         <v>0.17219999999999999</v>
       </c>
       <c r="F22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C23" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D23">
         <v>3</v>
       </c>
-      <c r="E23">
-        <v>43.5</v>
+      <c r="E23" t="s">
+        <v>72</v>
       </c>
       <c r="F23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C24" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D24">
         <v>4</v>
@@ -2577,18 +2751,18 @@
         <v>68</v>
       </c>
       <c r="F24" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B25" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D25">
         <v>5</v>
@@ -2597,7 +2771,7 @@
         <v>1000</v>
       </c>
       <c r="F25" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
@@ -2618,156 +2792,156 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
       <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
         <v>5</v>
-      </c>
-      <c r="E1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
         <v>30</v>
       </c>
-      <c r="C4" t="s">
-        <v>31</v>
-      </c>
       <c r="D4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" t="s">
         <v>30</v>
       </c>
-      <c r="C9" t="s">
-        <v>31</v>
-      </c>
       <c r="D9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -2777,83 +2951,68 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC6483DD-2255-49BA-BAE9-23EDEC3285E4}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.5" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" t="s">
         <v>36</v>
       </c>
-      <c r="B1" t="s">
-        <v>37</v>
-      </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="D1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" t="s">
         <v>49</v>
       </c>
-      <c r="C2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3">
+      <c r="C3">
         <v>100000</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" t="s">
         <v>68</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" t="s">
         <v>69</v>
       </c>
-      <c r="C4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B5" t="s">
-        <v>70</v>
-      </c>
-      <c r="C5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5">
+      <c r="C5">
         <v>100000</v>
       </c>
     </row>

</xml_diff>